<commit_message>
Improve how users access bid source information
Replace direct file path opening with a prioritized system for accessing bid origins, prioritizing BuildingConnected links, then file paths, and finally a disabled state.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1e5b925f-7248-4ca9-91c6-e89db97cd9e4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/yB3l5ea
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-12.xlsx
+++ b/backups/proposal-log-2026-04-12.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10604" uniqueCount="1270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10617" uniqueCount="1275">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -382,18 +382,48 @@
     <t>["Storefronts &amp; Curtain Walls"]</t>
   </si>
   <si>
+    <t>26-0211</t>
+  </si>
+  <si>
+    <t>Merci Keathley</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
+  </si>
+  <si>
+    <t>["69cc472c724d4f360623c300"]</t>
+  </si>
+  <si>
+    <t>["Appliances"]</t>
+  </si>
+  <si>
+    <t>26-0213</t>
+  </si>
+  <si>
+    <t>TRA General Office Complex</t>
+  </si>
+  <si>
+    <t>DFW</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>Christman Weeks</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
+  </si>
+  <si>
+    <t>["69ce6ad9ffa00f5f6b96a4d9"]</t>
+  </si>
+  <si>
     <t>26-0205</t>
   </si>
   <si>
-    <t>TRA General Office Complex</t>
-  </si>
-  <si>
-    <t>2026-04-02</t>
-  </si>
-  <si>
-    <t>2026-04-23</t>
-  </si>
-  <si>
     <t>Won</t>
   </si>
   <si>
@@ -403,36 +433,6 @@
     <t>2027-07-30</t>
   </si>
   <si>
-    <t>26-0213</t>
-  </si>
-  <si>
-    <t>DFW</t>
-  </si>
-  <si>
-    <t>Christman Weeks</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
-  </si>
-  <si>
-    <t>["69ce6ad9ffa00f5f6b96a4d9"]</t>
-  </si>
-  <si>
-    <t>26-0211</t>
-  </si>
-  <si>
-    <t>Merci Keathley</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
-  </si>
-  <si>
-    <t>["69cc472c724d4f360623c300"]</t>
-  </si>
-  <si>
-    <t>["Appliances"]</t>
-  </si>
-  <si>
     <t>26-0185</t>
   </si>
   <si>
@@ -697,6 +697,24 @@
     <t>26-0019</t>
   </si>
   <si>
+    <t>RB-26005</t>
+  </si>
+  <si>
+    <t>Market on morehead</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
+  </si>
+  <si>
+    <t>Louren Martinez</t>
+  </si>
+  <si>
+    <t>1783</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+  <si>
     <t>26-0215</t>
   </si>
   <si>
@@ -724,24 +742,6 @@
     <t>["Specialties &amp; Accessories"]</t>
   </si>
   <si>
-    <t>RB-26005</t>
-  </si>
-  <si>
-    <t>Market on morehead</t>
-  </si>
-  <si>
-    <t>2026-01-07</t>
-  </si>
-  <si>
-    <t>Louren Martinez</t>
-  </si>
-  <si>
-    <t>1783</t>
-  </si>
-  <si>
-    <t>2026-01-01</t>
-  </si>
-  <si>
     <t>RB-26023</t>
   </si>
   <si>
@@ -793,6 +793,39 @@
     <t>2028-02-01</t>
   </si>
   <si>
+    <t>26-0020</t>
+  </si>
+  <si>
+    <t>26-0196</t>
+  </si>
+  <si>
+    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Mark Socks</t>
+  </si>
+  <si>
+    <t>Lost</t>
+  </si>
+  <si>
+    <t>NO BID - No Scope</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
+  </si>
+  <si>
+    <t>["69c1b75e4cb9ae021994a5b7"]</t>
+  </si>
+  <si>
+    <t>["Expansion Control Systems"]</t>
+  </si>
+  <si>
     <t>26-0194</t>
   </si>
   <si>
@@ -817,7 +850,28 @@
     <t>QA Reviewer</t>
   </si>
   <si>
-    <t>26-0020</t>
+    <t>26-0200</t>
+  </si>
+  <si>
+    <t>Flying Pickle Idaho Falls</t>
+  </si>
+  <si>
+    <t>Washington (SEA)</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>["69cc01834e68f2d35d122b59"]</t>
+  </si>
+  <si>
+    <t>[]</t>
   </si>
   <si>
     <t>26-0214</t>
@@ -847,60 +901,6 @@
     <t>["2026-04-08T18:09:51.975Z: dueDate: 2026-04-07 → 2026-04-13"]</t>
   </si>
   <si>
-    <t>26-0200</t>
-  </si>
-  <si>
-    <t>Flying Pickle Idaho Falls</t>
-  </si>
-  <si>
-    <t>Washington (SEA)</t>
-  </si>
-  <si>
-    <t>2026-03-31</t>
-  </si>
-  <si>
-    <t>Jake Marrujo</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
-  </si>
-  <si>
-    <t>["69cc01834e68f2d35d122b59"]</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>26-0196</t>
-  </si>
-  <si>
-    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
-  </si>
-  <si>
-    <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>2026-04-07</t>
-  </si>
-  <si>
-    <t>Mark Socks</t>
-  </si>
-  <si>
-    <t>Lost</t>
-  </si>
-  <si>
-    <t>NO BID - No Scope</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
-  </si>
-  <si>
-    <t>["69c1b75e4cb9ae021994a5b7"]</t>
-  </si>
-  <si>
-    <t>["Expansion Control Systems"]</t>
-  </si>
-  <si>
     <t>26-0003</t>
   </si>
   <si>
@@ -1042,6 +1042,24 @@
     <t>1057256</t>
   </si>
   <si>
+    <t>26-0218</t>
+  </si>
+  <si>
+    <t>GoCary Bus Operations &amp; Maintenance Facility (BOMF)</t>
+  </si>
+  <si>
+    <t>CLT</t>
+  </si>
+  <si>
+    <t>DeShaun Taylor</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d3dce067942824a3512727</t>
+  </si>
+  <si>
+    <t>["69d3dce067942824a3512727"]</t>
+  </si>
+  <si>
     <t>ATL - Atlanta</t>
   </si>
   <si>
@@ -1093,24 +1111,6 @@
     <t>["Toilet Accessories","Wall Protection","FEC"]</t>
   </si>
   <si>
-    <t>26-0218</t>
-  </si>
-  <si>
-    <t>GoCary Bus Operations &amp; Maintenance Facility (BOMF)</t>
-  </si>
-  <si>
-    <t>CLT</t>
-  </si>
-  <si>
-    <t>DeShaun Taylor</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d3dce067942824a3512727</t>
-  </si>
-  <si>
-    <t>["69d3dce067942824a3512727"]</t>
-  </si>
-  <si>
     <t>26-0217</t>
   </si>
   <si>
@@ -1327,6 +1327,36 @@
     <t>1146456</t>
   </si>
   <si>
+    <t>26-0209</t>
+  </si>
+  <si>
+    <t>GEG</t>
+  </si>
+  <si>
+    <t>26-0208</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Gabriel Frota</t>
+  </si>
+  <si>
+    <t>10187</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
+  </si>
+  <si>
+    <t>["69c6f855787ef64d5cc05edb"]</t>
+  </si>
+  <si>
+    <t>["Sheet Metal &amp; Metal Panels"]</t>
+  </si>
+  <si>
     <t>26-0198</t>
   </si>
   <si>
@@ -1360,36 +1390,6 @@
     <t>["Flagpoles"]</t>
   </si>
   <si>
-    <t>26-0209</t>
-  </si>
-  <si>
-    <t>GEG</t>
-  </si>
-  <si>
-    <t>26-0208</t>
-  </si>
-  <si>
-    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
-  </si>
-  <si>
-    <t>Entertainment</t>
-  </si>
-  <si>
-    <t>Gabriel Frota</t>
-  </si>
-  <si>
-    <t>10187</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
-  </si>
-  <si>
-    <t>["69c6f855787ef64d5cc05edb"]</t>
-  </si>
-  <si>
-    <t>["Sheet Metal &amp; Metal Panels"]</t>
-  </si>
-  <si>
     <t>26-0028</t>
   </si>
   <si>
@@ -3553,6 +3553,15 @@
     <t>2026-04-09T04:10:45.117Z</t>
   </si>
   <si>
+    <t>2026-04-12T05:03:35.081Z</t>
+  </si>
+  <si>
+    <t>2026-04-12T05:05:23.018Z</t>
+  </si>
+  <si>
+    <t>2026-04-12T05:05:26.170Z</t>
+  </si>
+  <si>
     <t>fieldName</t>
   </si>
   <si>
@@ -3716,6 +3725,12 @@
   </si>
   <si>
     <t>2026-04-11T21:06:21.412Z</t>
+  </si>
+  <si>
+    <t>2026-04-12T05:04:46.450Z</t>
+  </si>
+  <si>
+    <t>2026-04-12T05:04:52.491Z</t>
   </si>
   <si>
     <t>bcOpportunityId</t>
@@ -5544,52 +5559,52 @@
         <v>122</v>
       </c>
       <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" t="s">
         <v>123</v>
       </c>
-      <c r="C13" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="I13" t="s">
+        <v>38</v>
+      </c>
+      <c r="J13" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" t="s">
+        <v>38</v>
+      </c>
+      <c r="L13" t="s">
+        <v>38</v>
+      </c>
+      <c r="M13" t="s">
+        <v>38</v>
+      </c>
+      <c r="N13" t="s">
         <v>124</v>
       </c>
-      <c r="F13" t="s">
-        <v>125</v>
-      </c>
-      <c r="G13" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" t="s">
-        <v>38</v>
-      </c>
-      <c r="J13" t="s">
-        <v>126</v>
-      </c>
-      <c r="K13" t="s">
-        <v>127</v>
-      </c>
-      <c r="L13" t="s">
-        <v>128</v>
-      </c>
-      <c r="M13" t="s">
-        <v>38</v>
-      </c>
-      <c r="N13" t="s">
-        <v>38</v>
-      </c>
       <c r="O13" t="s">
         <v>38</v>
       </c>
       <c r="P13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="Q13">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
@@ -5604,19 +5619,19 @@
         <v>38</v>
       </c>
       <c r="V13" t="s">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="W13" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="X13" t="s">
         <v>38</v>
       </c>
       <c r="Y13" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="Z13" s="2">
+        <v>46115.81093040509</v>
       </c>
       <c r="AA13" t="b">
         <v>0</v>
@@ -5643,33 +5658,33 @@
         <v>38</v>
       </c>
       <c r="AI13" s="2">
-        <v>46115.64971903936</v>
+        <v>46115.80864076389</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C14" t="s">
         <v>129</v>
-      </c>
-      <c r="B14" t="s">
-        <v>123</v>
-      </c>
-      <c r="C14" t="s">
-        <v>130</v>
       </c>
       <c r="D14" t="s">
         <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G14" t="s">
         <v>38</v>
       </c>
       <c r="H14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I14" t="s">
         <v>38</v>
@@ -5687,7 +5702,7 @@
         <v>38</v>
       </c>
       <c r="N14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O14" t="s">
         <v>38</v>
@@ -5711,7 +5726,7 @@
         <v>38</v>
       </c>
       <c r="V14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="W14" t="s">
         <v>57</v>
@@ -5755,55 +5770,55 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
-        <v>53</v>
+        <v>131</v>
       </c>
       <c r="G15" t="s">
         <v>38</v>
       </c>
       <c r="H15" t="s">
-        <v>135</v>
+        <v>38</v>
       </c>
       <c r="I15" t="s">
         <v>38</v>
       </c>
       <c r="J15" t="s">
-        <v>43</v>
+        <v>136</v>
       </c>
       <c r="K15" t="s">
-        <v>38</v>
+        <v>137</v>
       </c>
       <c r="L15" t="s">
-        <v>38</v>
+        <v>138</v>
       </c>
       <c r="M15" t="s">
         <v>38</v>
       </c>
       <c r="N15" t="s">
-        <v>136</v>
+        <v>38</v>
       </c>
       <c r="O15" t="s">
         <v>38</v>
       </c>
       <c r="P15" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q15">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="R15" t="b">
         <v>0</v>
@@ -5818,19 +5833,19 @@
         <v>38</v>
       </c>
       <c r="V15" t="s">
-        <v>137</v>
+        <v>38</v>
       </c>
       <c r="W15" t="s">
-        <v>138</v>
+        <v>38</v>
       </c>
       <c r="X15" t="s">
         <v>38</v>
       </c>
       <c r="Y15" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z15" s="2">
-        <v>46115.81093040509</v>
+        <v>38</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>38</v>
       </c>
       <c r="AA15" t="b">
         <v>0</v>
@@ -5857,7 +5872,7 @@
         <v>38</v>
       </c>
       <c r="AI15" s="2">
-        <v>46115.80864076389</v>
+        <v>46115.64971903936</v>
       </c>
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.25">
@@ -8115,49 +8130,49 @@
         <v>228</v>
       </c>
       <c r="C37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" t="s">
+        <v>155</v>
+      </c>
+      <c r="F37" t="s">
         <v>229</v>
       </c>
-      <c r="D37" t="s">
+      <c r="G37" t="s">
+        <v>151</v>
+      </c>
+      <c r="H37" t="s">
         <v>230</v>
       </c>
-      <c r="E37" t="s">
+      <c r="I37" t="s">
         <v>231</v>
       </c>
-      <c r="F37" t="s">
-        <v>144</v>
-      </c>
-      <c r="G37" t="s">
-        <v>38</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="J37" t="s">
+        <v>84</v>
+      </c>
+      <c r="K37" t="s">
         <v>232</v>
       </c>
-      <c r="I37" t="s">
-        <v>38</v>
-      </c>
-      <c r="J37" t="s">
-        <v>43</v>
-      </c>
-      <c r="K37" t="s">
-        <v>38</v>
-      </c>
       <c r="L37" t="s">
-        <v>38</v>
+        <v>232</v>
       </c>
       <c r="M37" t="s">
         <v>38</v>
       </c>
       <c r="N37" t="s">
-        <v>233</v>
+        <v>38</v>
       </c>
       <c r="O37" t="s">
         <v>38</v>
       </c>
       <c r="P37" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q37">
-        <v>109</v>
+        <v>38</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>38</v>
       </c>
       <c r="R37" t="b">
         <v>0</v>
@@ -8172,19 +8187,19 @@
         <v>38</v>
       </c>
       <c r="V37" t="s">
-        <v>234</v>
+        <v>38</v>
       </c>
       <c r="W37" t="s">
-        <v>235</v>
+        <v>38</v>
       </c>
       <c r="X37" t="s">
         <v>38</v>
       </c>
       <c r="Y37" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z37" s="2">
-        <v>46118.64171784722</v>
+        <v>38</v>
+      </c>
+      <c r="Z37" t="s">
+        <v>38</v>
       </c>
       <c r="AA37" t="b">
         <v>0</v>
@@ -8198,8 +8213,8 @@
       <c r="AD37" t="s">
         <v>38</v>
       </c>
-      <c r="AE37" t="s">
-        <v>38</v>
+      <c r="AE37" s="2">
+        <v>46111.1943433912</v>
       </c>
       <c r="AF37" t="b">
         <v>0</v>
@@ -8211,60 +8226,60 @@
         <v>38</v>
       </c>
       <c r="AI37" s="2">
-        <v>46118.63981587963</v>
+        <v>46101.831740231486</v>
       </c>
     </row>
     <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>233</v>
+      </c>
+      <c r="B38" t="s">
+        <v>234</v>
+      </c>
+      <c r="C38" t="s">
+        <v>235</v>
+      </c>
+      <c r="D38" t="s">
         <v>236</v>
       </c>
-      <c r="B38" t="s">
+      <c r="E38" t="s">
         <v>237</v>
       </c>
-      <c r="C38" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38" t="s">
-        <v>155</v>
-      </c>
       <c r="F38" t="s">
+        <v>144</v>
+      </c>
+      <c r="G38" t="s">
+        <v>69</v>
+      </c>
+      <c r="H38" t="s">
         <v>238</v>
       </c>
-      <c r="G38" t="s">
-        <v>151</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
+        <v>38</v>
+      </c>
+      <c r="J38" t="s">
+        <v>43</v>
+      </c>
+      <c r="K38" t="s">
+        <v>38</v>
+      </c>
+      <c r="L38" t="s">
+        <v>38</v>
+      </c>
+      <c r="M38" t="s">
+        <v>38</v>
+      </c>
+      <c r="N38" t="s">
         <v>239</v>
       </c>
-      <c r="I38" t="s">
-        <v>240</v>
-      </c>
-      <c r="J38" t="s">
-        <v>84</v>
-      </c>
-      <c r="K38" t="s">
-        <v>241</v>
-      </c>
-      <c r="L38" t="s">
-        <v>241</v>
-      </c>
-      <c r="M38" t="s">
-        <v>38</v>
-      </c>
-      <c r="N38" t="s">
-        <v>38</v>
-      </c>
       <c r="O38" t="s">
         <v>38</v>
       </c>
       <c r="P38" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>38</v>
+        <v>45</v>
+      </c>
+      <c r="Q38">
+        <v>109</v>
       </c>
       <c r="R38" t="b">
         <v>0</v>
@@ -8279,19 +8294,19 @@
         <v>38</v>
       </c>
       <c r="V38" t="s">
-        <v>38</v>
+        <v>240</v>
       </c>
       <c r="W38" t="s">
-        <v>38</v>
+        <v>241</v>
       </c>
       <c r="X38" t="s">
         <v>38</v>
       </c>
       <c r="Y38" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z38" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="Z38" s="2">
+        <v>46118.64171784722</v>
       </c>
       <c r="AA38" t="b">
         <v>0</v>
@@ -8305,8 +8320,8 @@
       <c r="AD38" t="s">
         <v>38</v>
       </c>
-      <c r="AE38" s="2">
-        <v>46111.1943433912</v>
+      <c r="AE38" t="s">
+        <v>38</v>
       </c>
       <c r="AF38" t="b">
         <v>0</v>
@@ -8318,7 +8333,7 @@
         <v>38</v>
       </c>
       <c r="AI38" s="2">
-        <v>46101.831740231486</v>
+        <v>46118.63981587963</v>
       </c>
     </row>
     <row r="39" spans="1:35" x14ac:dyDescent="0.25">
@@ -8546,7 +8561,7 @@
         <v>80</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="E41" t="s">
         <v>155</v>
@@ -8647,52 +8662,52 @@
         <v>259</v>
       </c>
       <c r="B42" t="s">
-        <v>260</v>
+        <v>172</v>
       </c>
       <c r="C42" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>200</v>
+        <v>52</v>
       </c>
       <c r="E42" t="s">
+        <v>173</v>
+      </c>
+      <c r="F42" t="s">
+        <v>174</v>
+      </c>
+      <c r="G42" t="s">
+        <v>151</v>
+      </c>
+      <c r="H42" t="s">
+        <v>38</v>
+      </c>
+      <c r="I42" t="s">
+        <v>38</v>
+      </c>
+      <c r="J42" t="s">
+        <v>43</v>
+      </c>
+      <c r="K42" t="s">
         <v>39</v>
       </c>
-      <c r="F42" t="s">
-        <v>210</v>
-      </c>
-      <c r="G42" t="s">
-        <v>38</v>
-      </c>
-      <c r="H42" t="s">
-        <v>261</v>
-      </c>
-      <c r="I42" t="s">
-        <v>262</v>
-      </c>
-      <c r="J42" t="s">
-        <v>84</v>
-      </c>
-      <c r="K42" t="s">
-        <v>38</v>
-      </c>
       <c r="L42" t="s">
-        <v>38</v>
+        <v>175</v>
       </c>
       <c r="M42" t="s">
         <v>38</v>
       </c>
       <c r="N42" t="s">
-        <v>263</v>
+        <v>38</v>
       </c>
       <c r="O42" t="s">
         <v>38</v>
       </c>
       <c r="P42" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q42">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="R42" t="b">
         <v>0</v>
@@ -8707,19 +8722,19 @@
         <v>38</v>
       </c>
       <c r="V42" t="s">
-        <v>264</v>
+        <v>38</v>
       </c>
       <c r="W42" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="X42" t="s">
-        <v>265</v>
+        <v>38</v>
       </c>
       <c r="Y42" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z42" s="2">
-        <v>46112.95053368056</v>
+        <v>38</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>38</v>
       </c>
       <c r="AA42" t="b">
         <v>0</v>
@@ -8728,13 +8743,13 @@
         <v>38</v>
       </c>
       <c r="AC42" t="s">
-        <v>266</v>
+        <v>38</v>
       </c>
       <c r="AD42" t="s">
         <v>38</v>
       </c>
-      <c r="AE42" t="s">
-        <v>38</v>
+      <c r="AE42" s="2">
+        <v>46093.859216736106</v>
       </c>
       <c r="AF42" t="b">
         <v>0</v>
@@ -8746,60 +8761,60 @@
         <v>38</v>
       </c>
       <c r="AI42" s="2">
-        <v>46112.94978048611</v>
+        <v>46093.82415605324</v>
       </c>
     </row>
     <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>260</v>
+      </c>
+      <c r="B43" t="s">
+        <v>261</v>
+      </c>
+      <c r="C43" t="s">
+        <v>235</v>
+      </c>
+      <c r="D43" t="s">
+        <v>38</v>
+      </c>
+      <c r="E43" t="s">
+        <v>262</v>
+      </c>
+      <c r="F43" t="s">
+        <v>263</v>
+      </c>
+      <c r="G43" t="s">
+        <v>38</v>
+      </c>
+      <c r="H43" t="s">
+        <v>264</v>
+      </c>
+      <c r="I43" t="s">
+        <v>38</v>
+      </c>
+      <c r="J43" t="s">
+        <v>265</v>
+      </c>
+      <c r="K43" t="s">
+        <v>38</v>
+      </c>
+      <c r="L43" t="s">
+        <v>38</v>
+      </c>
+      <c r="M43" t="s">
+        <v>266</v>
+      </c>
+      <c r="N43" t="s">
         <v>267</v>
       </c>
-      <c r="B43" t="s">
-        <v>172</v>
-      </c>
-      <c r="C43" t="s">
-        <v>73</v>
-      </c>
-      <c r="D43" t="s">
-        <v>52</v>
-      </c>
-      <c r="E43" t="s">
-        <v>173</v>
-      </c>
-      <c r="F43" t="s">
-        <v>174</v>
-      </c>
-      <c r="G43" t="s">
-        <v>151</v>
-      </c>
-      <c r="H43" t="s">
-        <v>38</v>
-      </c>
-      <c r="I43" t="s">
-        <v>38</v>
-      </c>
-      <c r="J43" t="s">
-        <v>43</v>
-      </c>
-      <c r="K43" t="s">
-        <v>39</v>
-      </c>
-      <c r="L43" t="s">
-        <v>175</v>
-      </c>
-      <c r="M43" t="s">
-        <v>38</v>
-      </c>
-      <c r="N43" t="s">
-        <v>38</v>
-      </c>
       <c r="O43" t="s">
         <v>38</v>
       </c>
       <c r="P43" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="Q43">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="R43" t="b">
         <v>0</v>
@@ -8814,19 +8829,19 @@
         <v>38</v>
       </c>
       <c r="V43" t="s">
-        <v>38</v>
+        <v>268</v>
       </c>
       <c r="W43" t="s">
-        <v>38</v>
+        <v>269</v>
       </c>
       <c r="X43" t="s">
         <v>38</v>
       </c>
       <c r="Y43" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z43" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="Z43" s="2">
+        <v>46112.951310543984</v>
       </c>
       <c r="AA43" t="b">
         <v>0</v>
@@ -8840,8 +8855,8 @@
       <c r="AD43" t="s">
         <v>38</v>
       </c>
-      <c r="AE43" s="2">
-        <v>46093.859216736106</v>
+      <c r="AE43" t="s">
+        <v>38</v>
       </c>
       <c r="AF43" t="b">
         <v>0</v>
@@ -8853,39 +8868,39 @@
         <v>38</v>
       </c>
       <c r="AI43" s="2">
-        <v>46093.82415605324</v>
+        <v>46112.94978027778</v>
       </c>
     </row>
     <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B44" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C44" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="D44" t="s">
-        <v>38</v>
+        <v>200</v>
       </c>
       <c r="E44" t="s">
-        <v>231</v>
+        <v>39</v>
       </c>
       <c r="F44" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G44" t="s">
         <v>38</v>
       </c>
       <c r="H44" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I44" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="J44" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="K44" t="s">
         <v>38</v>
@@ -8897,7 +8912,7 @@
         <v>38</v>
       </c>
       <c r="N44" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="O44" t="s">
         <v>38</v>
@@ -8906,7 +8921,7 @@
         <v>45</v>
       </c>
       <c r="Q44">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="R44" t="b">
         <v>0</v>
@@ -8921,28 +8936,28 @@
         <v>38</v>
       </c>
       <c r="V44" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="W44" t="s">
-        <v>274</v>
+        <v>57</v>
       </c>
       <c r="X44" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Y44" t="s">
         <v>48</v>
       </c>
       <c r="Z44" s="2">
-        <v>46115.811258125</v>
+        <v>46112.95053368056</v>
       </c>
       <c r="AA44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB44" t="s">
-        <v>276</v>
+        <v>38</v>
       </c>
       <c r="AC44" t="s">
-        <v>38</v>
+        <v>277</v>
       </c>
       <c r="AD44" t="s">
         <v>38</v>
@@ -8960,24 +8975,24 @@
         <v>38</v>
       </c>
       <c r="AI44" s="2">
-        <v>46115.80863989583</v>
+        <v>46112.94978048611</v>
       </c>
     </row>
     <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B45" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C45" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D45" t="s">
         <v>52</v>
       </c>
       <c r="E45" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F45" t="s">
         <v>218</v>
@@ -8986,7 +9001,7 @@
         <v>38</v>
       </c>
       <c r="H45" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I45" t="s">
         <v>38</v>
@@ -9004,7 +9019,7 @@
         <v>38</v>
       </c>
       <c r="N45" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="O45" t="s">
         <v>38</v>
@@ -9028,13 +9043,13 @@
         <v>38</v>
       </c>
       <c r="V45" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="W45" t="s">
         <v>57</v>
       </c>
       <c r="X45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Y45" t="s">
         <v>48</v>
@@ -9072,46 +9087,46 @@
     </row>
     <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B46" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C46" t="s">
-        <v>229</v>
+        <v>51</v>
       </c>
       <c r="D46" t="s">
         <v>38</v>
       </c>
       <c r="E46" t="s">
-        <v>287</v>
+        <v>237</v>
       </c>
       <c r="F46" t="s">
+        <v>218</v>
+      </c>
+      <c r="G46" t="s">
+        <v>38</v>
+      </c>
+      <c r="H46" t="s">
         <v>288</v>
       </c>
-      <c r="G46" t="s">
-        <v>38</v>
-      </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>289</v>
       </c>
-      <c r="I46" t="s">
-        <v>38</v>
-      </c>
       <c r="J46" t="s">
+        <v>43</v>
+      </c>
+      <c r="K46" t="s">
+        <v>38</v>
+      </c>
+      <c r="L46" t="s">
+        <v>38</v>
+      </c>
+      <c r="M46" t="s">
+        <v>38</v>
+      </c>
+      <c r="N46" t="s">
         <v>290</v>
-      </c>
-      <c r="K46" t="s">
-        <v>38</v>
-      </c>
-      <c r="L46" t="s">
-        <v>38</v>
-      </c>
-      <c r="M46" t="s">
-        <v>291</v>
-      </c>
-      <c r="N46" t="s">
-        <v>292</v>
       </c>
       <c r="O46" t="s">
         <v>38</v>
@@ -9120,7 +9135,7 @@
         <v>45</v>
       </c>
       <c r="Q46">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="R46" t="b">
         <v>0</v>
@@ -9135,25 +9150,25 @@
         <v>38</v>
       </c>
       <c r="V46" t="s">
+        <v>291</v>
+      </c>
+      <c r="W46" t="s">
+        <v>292</v>
+      </c>
+      <c r="X46" t="s">
         <v>293</v>
-      </c>
-      <c r="W46" t="s">
-        <v>294</v>
-      </c>
-      <c r="X46" t="s">
-        <v>38</v>
       </c>
       <c r="Y46" t="s">
         <v>48</v>
       </c>
       <c r="Z46" s="2">
-        <v>46112.951310543984</v>
+        <v>46115.811258125</v>
       </c>
       <c r="AA46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB46" t="s">
-        <v>38</v>
+        <v>294</v>
       </c>
       <c r="AC46" t="s">
         <v>38</v>
@@ -9174,7 +9189,7 @@
         <v>38</v>
       </c>
       <c r="AI46" s="2">
-        <v>46112.94978027778</v>
+        <v>46115.80863989583</v>
       </c>
     </row>
     <row r="47" spans="1:35" x14ac:dyDescent="0.25">
@@ -10463,34 +10478,34 @@
     </row>
     <row r="59" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>38</v>
+        <v>342</v>
       </c>
       <c r="B59" t="s">
-        <v>50</v>
+        <v>343</v>
       </c>
       <c r="C59" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D59" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E59" t="s">
-        <v>39</v>
+        <v>210</v>
       </c>
       <c r="F59" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="G59" t="s">
         <v>69</v>
       </c>
       <c r="H59" t="s">
-        <v>135</v>
+        <v>345</v>
       </c>
       <c r="I59" t="s">
         <v>38</v>
       </c>
       <c r="J59" t="s">
-        <v>343</v>
+        <v>43</v>
       </c>
       <c r="K59" t="s">
         <v>38</v>
@@ -10502,16 +10517,16 @@
         <v>38</v>
       </c>
       <c r="N59" t="s">
-        <v>136</v>
+        <v>346</v>
       </c>
       <c r="O59" t="s">
-        <v>344</v>
+        <v>38</v>
       </c>
       <c r="P59" t="s">
         <v>45</v>
       </c>
-      <c r="Q59" t="s">
-        <v>38</v>
+      <c r="Q59">
+        <v>112</v>
       </c>
       <c r="R59" t="b">
         <v>0</v>
@@ -10526,25 +10541,25 @@
         <v>38</v>
       </c>
       <c r="V59" t="s">
-        <v>137</v>
+        <v>347</v>
       </c>
       <c r="W59" t="s">
-        <v>138</v>
+        <v>57</v>
       </c>
       <c r="X59" t="s">
         <v>38</v>
       </c>
       <c r="Y59" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z59" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="Z59" s="2">
+        <v>46120.75758967592</v>
       </c>
       <c r="AA59" t="b">
         <v>0</v>
       </c>
       <c r="AB59" t="s">
-        <v>345</v>
+        <v>38</v>
       </c>
       <c r="AC59" t="s">
         <v>38</v>
@@ -10552,8 +10567,8 @@
       <c r="AD59" t="s">
         <v>38</v>
       </c>
-      <c r="AE59" s="2">
-        <v>46114.95109008102</v>
+      <c r="AE59" t="s">
+        <v>38</v>
       </c>
       <c r="AF59" t="b">
         <v>0</v>
@@ -10565,39 +10580,39 @@
         <v>38</v>
       </c>
       <c r="AI59" s="2">
-        <v>46113.82840027778</v>
+        <v>46120.75685143519</v>
       </c>
     </row>
     <row r="60" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>346</v>
+        <v>38</v>
       </c>
       <c r="B60" t="s">
-        <v>269</v>
+        <v>50</v>
       </c>
       <c r="C60" t="s">
-        <v>38</v>
+        <v>348</v>
       </c>
       <c r="D60" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="E60" t="s">
-        <v>347</v>
+        <v>39</v>
       </c>
       <c r="F60" t="s">
-        <v>288</v>
+        <v>53</v>
       </c>
       <c r="G60" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H60" t="s">
-        <v>270</v>
+        <v>123</v>
       </c>
       <c r="I60" t="s">
         <v>38</v>
       </c>
       <c r="J60" t="s">
-        <v>43</v>
+        <v>349</v>
       </c>
       <c r="K60" t="s">
         <v>38</v>
@@ -10609,16 +10624,16 @@
         <v>38</v>
       </c>
       <c r="N60" t="s">
-        <v>348</v>
+        <v>124</v>
       </c>
       <c r="O60" t="s">
-        <v>38</v>
+        <v>350</v>
       </c>
       <c r="P60" t="s">
         <v>45</v>
       </c>
-      <c r="Q60">
-        <v>90</v>
+      <c r="Q60" t="s">
+        <v>38</v>
       </c>
       <c r="R60" t="b">
         <v>0</v>
@@ -10633,25 +10648,25 @@
         <v>38</v>
       </c>
       <c r="V60" t="s">
-        <v>349</v>
+        <v>125</v>
       </c>
       <c r="W60" t="s">
-        <v>57</v>
+        <v>126</v>
       </c>
       <c r="X60" t="s">
-        <v>350</v>
+        <v>38</v>
       </c>
       <c r="Y60" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z60" s="2">
-        <v>46112.951018148146</v>
+        <v>38</v>
+      </c>
+      <c r="Z60" t="s">
+        <v>38</v>
       </c>
       <c r="AA60" t="b">
         <v>0</v>
       </c>
       <c r="AB60" t="s">
-        <v>38</v>
+        <v>351</v>
       </c>
       <c r="AC60" t="s">
         <v>38</v>
@@ -10660,7 +10675,7 @@
         <v>38</v>
       </c>
       <c r="AE60" s="2">
-        <v>46113.94965768518</v>
+        <v>46114.95109008102</v>
       </c>
       <c r="AF60" t="b">
         <v>0</v>
@@ -10672,36 +10687,36 @@
         <v>38</v>
       </c>
       <c r="AI60" s="2">
-        <v>46112.94978038194</v>
+        <v>46113.82840027778</v>
       </c>
     </row>
     <row r="61" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B61" t="s">
-        <v>352</v>
+        <v>287</v>
       </c>
       <c r="C61" t="s">
-        <v>130</v>
+        <v>38</v>
       </c>
       <c r="D61" t="s">
         <v>52</v>
       </c>
       <c r="E61" t="s">
+        <v>353</v>
+      </c>
+      <c r="F61" t="s">
+        <v>263</v>
+      </c>
+      <c r="G61" t="s">
+        <v>38</v>
+      </c>
+      <c r="H61" t="s">
         <v>288</v>
       </c>
-      <c r="F61" t="s">
-        <v>353</v>
-      </c>
-      <c r="G61" t="s">
-        <v>116</v>
-      </c>
-      <c r="H61" t="s">
-        <v>354</v>
-      </c>
       <c r="I61" t="s">
-        <v>355</v>
+        <v>38</v>
       </c>
       <c r="J61" t="s">
         <v>43</v>
@@ -10716,7 +10731,7 @@
         <v>38</v>
       </c>
       <c r="N61" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="O61" t="s">
         <v>38</v>
@@ -10725,7 +10740,7 @@
         <v>45</v>
       </c>
       <c r="Q61">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="R61" t="b">
         <v>0</v>
@@ -10740,19 +10755,19 @@
         <v>38</v>
       </c>
       <c r="V61" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="W61" t="s">
         <v>57</v>
       </c>
       <c r="X61" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="Y61" t="s">
         <v>48</v>
       </c>
       <c r="Z61" s="2">
-        <v>46120.75803053241</v>
+        <v>46112.951018148146</v>
       </c>
       <c r="AA61" t="b">
         <v>0</v>
@@ -10766,8 +10781,8 @@
       <c r="AD61" t="s">
         <v>38</v>
       </c>
-      <c r="AE61" t="s">
-        <v>38</v>
+      <c r="AE61" s="2">
+        <v>46113.94965768518</v>
       </c>
       <c r="AF61" t="b">
         <v>0</v>
@@ -10779,36 +10794,36 @@
         <v>38</v>
       </c>
       <c r="AI61" s="2">
-        <v>46120.756850844904</v>
+        <v>46112.94978038194</v>
       </c>
     </row>
     <row r="62" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B62" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C62" t="s">
-        <v>361</v>
+        <v>129</v>
       </c>
       <c r="D62" t="s">
         <v>52</v>
       </c>
       <c r="E62" t="s">
-        <v>210</v>
+        <v>263</v>
       </c>
       <c r="F62" t="s">
-        <v>103</v>
+        <v>359</v>
       </c>
       <c r="G62" t="s">
-        <v>38</v>
+        <v>116</v>
       </c>
       <c r="H62" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I62" t="s">
-        <v>38</v>
+        <v>361</v>
       </c>
       <c r="J62" t="s">
         <v>43</v>
@@ -10823,7 +10838,7 @@
         <v>38</v>
       </c>
       <c r="N62" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="O62" t="s">
         <v>38</v>
@@ -10832,7 +10847,7 @@
         <v>45</v>
       </c>
       <c r="Q62">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R62" t="b">
         <v>0</v>
@@ -10847,19 +10862,19 @@
         <v>38</v>
       </c>
       <c r="V62" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="W62" t="s">
         <v>57</v>
       </c>
       <c r="X62" t="s">
-        <v>38</v>
+        <v>364</v>
       </c>
       <c r="Y62" t="s">
         <v>48</v>
       </c>
       <c r="Z62" s="2">
-        <v>46120.75758967592</v>
+        <v>46120.75803053241</v>
       </c>
       <c r="AA62" t="b">
         <v>0</v>
@@ -10886,7 +10901,7 @@
         <v>38</v>
       </c>
       <c r="AI62" s="2">
-        <v>46120.75685143519</v>
+        <v>46120.756850844904</v>
       </c>
     </row>
     <row r="63" spans="1:35" x14ac:dyDescent="0.25">
@@ -10894,10 +10909,10 @@
         <v>365</v>
       </c>
       <c r="B63" t="s">
-        <v>360</v>
+        <v>343</v>
       </c>
       <c r="C63" t="s">
-        <v>361</v>
+        <v>344</v>
       </c>
       <c r="D63" t="s">
         <v>52</v>
@@ -10912,7 +10927,7 @@
         <v>366</v>
       </c>
       <c r="H63" t="s">
-        <v>362</v>
+        <v>345</v>
       </c>
       <c r="I63" t="s">
         <v>38</v>
@@ -11120,7 +11135,7 @@
         <v>53</v>
       </c>
       <c r="F65" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G65" t="s">
         <v>38</v>
@@ -11539,7 +11554,7 @@
         <v>397</v>
       </c>
       <c r="C69" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D69" t="s">
         <v>52</v>
@@ -11548,7 +11563,7 @@
         <v>185</v>
       </c>
       <c r="F69" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G69" t="s">
         <v>38</v>
@@ -11646,7 +11661,7 @@
         <v>399</v>
       </c>
       <c r="C70" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D70" t="s">
         <v>94</v>
@@ -12074,7 +12089,7 @@
         <v>415</v>
       </c>
       <c r="C74" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D74" t="s">
         <v>52</v>
@@ -12083,7 +12098,7 @@
         <v>155</v>
       </c>
       <c r="F74" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G74" t="s">
         <v>116</v>
@@ -12205,7 +12220,7 @@
         <v>84</v>
       </c>
       <c r="K75" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="L75" t="s">
         <v>424</v>
@@ -12606,7 +12621,7 @@
         <v>437</v>
       </c>
       <c r="B79" t="s">
-        <v>100</v>
+        <v>279</v>
       </c>
       <c r="C79" t="s">
         <v>438</v>
@@ -12615,16 +12630,16 @@
         <v>52</v>
       </c>
       <c r="E79" t="s">
-        <v>102</v>
+        <v>281</v>
       </c>
       <c r="F79" t="s">
-        <v>103</v>
+        <v>218</v>
       </c>
       <c r="G79" t="s">
-        <v>38</v>
+        <v>366</v>
       </c>
       <c r="H79" t="s">
-        <v>104</v>
+        <v>282</v>
       </c>
       <c r="I79" t="s">
         <v>38</v>
@@ -12642,7 +12657,7 @@
         <v>38</v>
       </c>
       <c r="N79" t="s">
-        <v>107</v>
+        <v>283</v>
       </c>
       <c r="O79" t="s">
         <v>38</v>
@@ -12651,7 +12666,7 @@
         <v>45</v>
       </c>
       <c r="Q79">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="R79" t="b">
         <v>0</v>
@@ -12666,7 +12681,7 @@
         <v>38</v>
       </c>
       <c r="V79" t="s">
-        <v>108</v>
+        <v>284</v>
       </c>
       <c r="W79" t="s">
         <v>57</v>
@@ -12678,7 +12693,7 @@
         <v>48</v>
       </c>
       <c r="Z79" s="2">
-        <v>46112.95175853009</v>
+        <v>46115.81067839121</v>
       </c>
       <c r="AA79" t="b">
         <v>0</v>
@@ -12692,8 +12707,8 @@
       <c r="AD79" t="s">
         <v>38</v>
       </c>
-      <c r="AE79" s="2">
-        <v>46113.94965768518</v>
+      <c r="AE79" t="s">
+        <v>38</v>
       </c>
       <c r="AF79" t="b">
         <v>0</v>
@@ -12705,7 +12720,7 @@
         <v>38</v>
       </c>
       <c r="AI79" s="2">
-        <v>46112.94978008102</v>
+        <v>46115.808641111114</v>
       </c>
     </row>
     <row r="80" spans="1:35" x14ac:dyDescent="0.25">
@@ -12713,28 +12728,28 @@
         <v>439</v>
       </c>
       <c r="B80" t="s">
-        <v>111</v>
+        <v>440</v>
       </c>
       <c r="C80" t="s">
-        <v>440</v>
+        <v>112</v>
       </c>
       <c r="D80" t="s">
-        <v>113</v>
+        <v>441</v>
       </c>
       <c r="E80" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="F80" t="s">
-        <v>115</v>
+        <v>262</v>
       </c>
       <c r="G80" t="s">
-        <v>38</v>
+        <v>116</v>
       </c>
       <c r="H80" t="s">
-        <v>117</v>
+        <v>442</v>
       </c>
       <c r="I80" t="s">
-        <v>38</v>
+        <v>443</v>
       </c>
       <c r="J80" t="s">
         <v>43</v>
@@ -12749,7 +12764,7 @@
         <v>38</v>
       </c>
       <c r="N80" t="s">
-        <v>119</v>
+        <v>444</v>
       </c>
       <c r="O80" t="s">
         <v>38</v>
@@ -12758,7 +12773,7 @@
         <v>45</v>
       </c>
       <c r="Q80">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="R80" t="b">
         <v>0</v>
@@ -12773,25 +12788,25 @@
         <v>38</v>
       </c>
       <c r="V80" t="s">
-        <v>120</v>
+        <v>445</v>
       </c>
       <c r="W80" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="X80" t="s">
-        <v>442</v>
+        <v>109</v>
       </c>
       <c r="Y80" t="s">
         <v>48</v>
       </c>
       <c r="Z80" s="2">
-        <v>46112.951662962965</v>
+        <v>46115.810453784725</v>
       </c>
       <c r="AA80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB80" t="s">
-        <v>443</v>
+        <v>38</v>
       </c>
       <c r="AC80" t="s">
         <v>38</v>
@@ -12799,8 +12814,8 @@
       <c r="AD80" t="s">
         <v>38</v>
       </c>
-      <c r="AE80" s="2">
-        <v>46113.94965768518</v>
+      <c r="AE80" t="s">
+        <v>38</v>
       </c>
       <c r="AF80" t="b">
         <v>0</v>
@@ -12812,24 +12827,24 @@
         <v>38</v>
       </c>
       <c r="AI80" s="2">
-        <v>46112.949780173614</v>
+        <v>46115.80864127315</v>
       </c>
     </row>
     <row r="81" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B81" t="s">
-        <v>360</v>
+        <v>100</v>
       </c>
       <c r="C81" t="s">
-        <v>361</v>
+        <v>448</v>
       </c>
       <c r="D81" t="s">
         <v>52</v>
       </c>
       <c r="E81" t="s">
-        <v>210</v>
+        <v>102</v>
       </c>
       <c r="F81" t="s">
         <v>103</v>
@@ -12838,10 +12853,10 @@
         <v>38</v>
       </c>
       <c r="H81" t="s">
-        <v>362</v>
+        <v>104</v>
       </c>
       <c r="I81" t="s">
-        <v>271</v>
+        <v>38</v>
       </c>
       <c r="J81" t="s">
         <v>43</v>
@@ -12856,7 +12871,7 @@
         <v>38</v>
       </c>
       <c r="N81" t="s">
-        <v>445</v>
+        <v>107</v>
       </c>
       <c r="O81" t="s">
         <v>38</v>
@@ -12865,7 +12880,7 @@
         <v>45</v>
       </c>
       <c r="Q81">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="R81" t="b">
         <v>0</v>
@@ -12880,10 +12895,10 @@
         <v>38</v>
       </c>
       <c r="V81" t="s">
-        <v>446</v>
+        <v>108</v>
       </c>
       <c r="W81" t="s">
-        <v>447</v>
+        <v>57</v>
       </c>
       <c r="X81" t="s">
         <v>38</v>
@@ -12892,7 +12907,7 @@
         <v>48</v>
       </c>
       <c r="Z81" s="2">
-        <v>46118.958962268516</v>
+        <v>46112.95175853009</v>
       </c>
       <c r="AA81" t="b">
         <v>0</v>
@@ -12907,45 +12922,45 @@
         <v>38</v>
       </c>
       <c r="AE81" s="2">
-        <v>46121.252319861116</v>
+        <v>46113.94965768518</v>
       </c>
       <c r="AF81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG81" t="s">
-        <v>69</v>
-      </c>
-      <c r="AH81" s="2">
-        <v>46121.25048729166</v>
+        <v>38</v>
+      </c>
+      <c r="AH81" t="s">
+        <v>38</v>
       </c>
       <c r="AI81" s="2">
-        <v>46118.957825254634</v>
+        <v>46112.94978008102</v>
       </c>
     </row>
     <row r="82" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B82" t="s">
-        <v>278</v>
+        <v>111</v>
       </c>
       <c r="C82" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D82" t="s">
-        <v>52</v>
+        <v>113</v>
       </c>
       <c r="E82" t="s">
-        <v>280</v>
+        <v>114</v>
       </c>
       <c r="F82" t="s">
-        <v>218</v>
+        <v>115</v>
       </c>
       <c r="G82" t="s">
-        <v>366</v>
+        <v>38</v>
       </c>
       <c r="H82" t="s">
-        <v>281</v>
+        <v>117</v>
       </c>
       <c r="I82" t="s">
         <v>38</v>
@@ -12963,7 +12978,7 @@
         <v>38</v>
       </c>
       <c r="N82" t="s">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="O82" t="s">
         <v>38</v>
@@ -12972,7 +12987,7 @@
         <v>45</v>
       </c>
       <c r="Q82">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="R82" t="b">
         <v>0</v>
@@ -12987,25 +13002,25 @@
         <v>38</v>
       </c>
       <c r="V82" t="s">
-        <v>283</v>
+        <v>120</v>
       </c>
       <c r="W82" t="s">
-        <v>57</v>
+        <v>451</v>
       </c>
       <c r="X82" t="s">
-        <v>38</v>
+        <v>452</v>
       </c>
       <c r="Y82" t="s">
         <v>48</v>
       </c>
       <c r="Z82" s="2">
-        <v>46115.81067839121</v>
+        <v>46112.951662962965</v>
       </c>
       <c r="AA82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB82" t="s">
-        <v>38</v>
+        <v>453</v>
       </c>
       <c r="AC82" t="s">
         <v>38</v>
@@ -13013,8 +13028,8 @@
       <c r="AD82" t="s">
         <v>38</v>
       </c>
-      <c r="AE82" t="s">
-        <v>38</v>
+      <c r="AE82" s="2">
+        <v>46113.94965768518</v>
       </c>
       <c r="AF82" t="b">
         <v>0</v>
@@ -13026,36 +13041,36 @@
         <v>38</v>
       </c>
       <c r="AI82" s="2">
-        <v>46115.808641111114</v>
+        <v>46112.949780173614</v>
       </c>
     </row>
     <row r="83" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B83" t="s">
-        <v>451</v>
+        <v>343</v>
       </c>
       <c r="C83" t="s">
-        <v>112</v>
+        <v>344</v>
       </c>
       <c r="D83" t="s">
-        <v>452</v>
+        <v>52</v>
       </c>
       <c r="E83" t="s">
-        <v>102</v>
+        <v>210</v>
       </c>
       <c r="F83" t="s">
-        <v>287</v>
+        <v>103</v>
       </c>
       <c r="G83" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="H83" t="s">
-        <v>453</v>
+        <v>345</v>
       </c>
       <c r="I83" t="s">
-        <v>454</v>
+        <v>289</v>
       </c>
       <c r="J83" t="s">
         <v>43</v>
@@ -13079,7 +13094,7 @@
         <v>45</v>
       </c>
       <c r="Q83">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="R83" t="b">
         <v>0</v>
@@ -13100,13 +13115,13 @@
         <v>457</v>
       </c>
       <c r="X83" t="s">
-        <v>109</v>
+        <v>38</v>
       </c>
       <c r="Y83" t="s">
         <v>48</v>
       </c>
       <c r="Z83" s="2">
-        <v>46115.810453784725</v>
+        <v>46118.958962268516</v>
       </c>
       <c r="AA83" t="b">
         <v>0</v>
@@ -13120,20 +13135,20 @@
       <c r="AD83" t="s">
         <v>38</v>
       </c>
-      <c r="AE83" t="s">
-        <v>38</v>
+      <c r="AE83" s="2">
+        <v>46121.252319861116</v>
       </c>
       <c r="AF83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG83" t="s">
-        <v>38</v>
-      </c>
-      <c r="AH83" t="s">
-        <v>38</v>
+        <v>69</v>
+      </c>
+      <c r="AH83" s="2">
+        <v>46121.25048729166</v>
       </c>
       <c r="AI83" s="2">
-        <v>46115.80864127315</v>
+        <v>46118.957825254634</v>
       </c>
     </row>
     <row r="84" spans="1:35" x14ac:dyDescent="0.25">
@@ -13260,7 +13275,7 @@
         <v>155</v>
       </c>
       <c r="F85" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G85" t="s">
         <v>116</v>
@@ -13367,7 +13382,7 @@
         <v>155</v>
       </c>
       <c r="F86" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G86" t="s">
         <v>116</v>
@@ -13896,7 +13911,7 @@
         <v>217</v>
       </c>
       <c r="D91" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E91" t="s">
         <v>155</v>
@@ -14122,7 +14137,7 @@
         <v>38</v>
       </c>
       <c r="H93" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="I93" t="s">
         <v>38</v>
@@ -14211,7 +14226,7 @@
         <v>502</v>
       </c>
       <c r="B94" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="C94" t="s">
         <v>112</v>
@@ -14223,13 +14238,13 @@
         <v>102</v>
       </c>
       <c r="F94" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G94" t="s">
         <v>38</v>
       </c>
       <c r="H94" t="s">
-        <v>453</v>
+        <v>442</v>
       </c>
       <c r="I94" t="s">
         <v>38</v>
@@ -14247,7 +14262,7 @@
         <v>504</v>
       </c>
       <c r="N94" t="s">
-        <v>455</v>
+        <v>444</v>
       </c>
       <c r="O94" t="s">
         <v>38</v>
@@ -14271,10 +14286,10 @@
         <v>38</v>
       </c>
       <c r="V94" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
       <c r="W94" t="s">
-        <v>457</v>
+        <v>446</v>
       </c>
       <c r="X94" t="s">
         <v>505</v>
@@ -14749,10 +14764,10 @@
         <v>524</v>
       </c>
       <c r="C99" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D99" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E99" t="s">
         <v>174</v>
@@ -14972,7 +14987,7 @@
         <v>155</v>
       </c>
       <c r="F101" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G101" t="s">
         <v>151</v>
@@ -15709,7 +15724,7 @@
         <v>555</v>
       </c>
       <c r="B108" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C108" t="s">
         <v>38</v>
@@ -15718,22 +15733,22 @@
         <v>66</v>
       </c>
       <c r="E108" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F108" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="G108" t="s">
         <v>38</v>
       </c>
       <c r="H108" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I108" t="s">
         <v>38</v>
       </c>
       <c r="J108" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="K108" t="s">
         <v>38</v>
@@ -15745,7 +15760,7 @@
         <v>38</v>
       </c>
       <c r="N108" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O108" t="s">
         <v>38</v>
@@ -15769,7 +15784,7 @@
         <v>38</v>
       </c>
       <c r="V108" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="W108" t="s">
         <v>57</v>
@@ -15929,7 +15944,7 @@
         <v>299</v>
       </c>
       <c r="D110" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E110" t="s">
         <v>155</v>
@@ -16149,7 +16164,7 @@
         <v>155</v>
       </c>
       <c r="F112" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G112" t="s">
         <v>116</v>
@@ -16470,7 +16485,7 @@
         <v>194</v>
       </c>
       <c r="F115" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G115" t="s">
         <v>69</v>
@@ -16678,7 +16693,7 @@
         <v>149</v>
       </c>
       <c r="D117" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E117" t="s">
         <v>155</v>
@@ -16889,7 +16904,7 @@
         <v>587</v>
       </c>
       <c r="C119" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D119" t="s">
         <v>142</v>
@@ -16904,7 +16919,7 @@
         <v>116</v>
       </c>
       <c r="H119" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="I119" t="s">
         <v>588</v>
@@ -17852,7 +17867,7 @@
         <v>399</v>
       </c>
       <c r="C128" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D128" t="s">
         <v>94</v>
@@ -20741,7 +20756,7 @@
         <v>704</v>
       </c>
       <c r="C155" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D155" t="s">
         <v>52</v>
@@ -22563,7 +22578,7 @@
         <v>221</v>
       </c>
       <c r="D172" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E172" t="s">
         <v>155</v>
@@ -23630,7 +23645,7 @@
         <v>785</v>
       </c>
       <c r="C182" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D182" t="s">
         <v>52</v>
@@ -23639,7 +23654,7 @@
         <v>194</v>
       </c>
       <c r="F182" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="G182" t="s">
         <v>69</v>
@@ -23844,7 +23859,7 @@
         <v>792</v>
       </c>
       <c r="C184" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D184" t="s">
         <v>52</v>
@@ -23859,7 +23874,7 @@
         <v>69</v>
       </c>
       <c r="H184" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="I184" t="s">
         <v>793</v>
@@ -25770,7 +25785,7 @@
         <v>856</v>
       </c>
       <c r="C202" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D202" t="s">
         <v>142</v>
@@ -26849,7 +26864,7 @@
         <v>155</v>
       </c>
       <c r="F212" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="G212" t="s">
         <v>38</v>
@@ -27378,7 +27393,7 @@
         <v>149</v>
       </c>
       <c r="D217" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E217" t="s">
         <v>155</v>
@@ -27598,7 +27613,7 @@
         <v>155</v>
       </c>
       <c r="F219" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G219" t="s">
         <v>116</v>
@@ -27699,13 +27714,13 @@
         <v>303</v>
       </c>
       <c r="D220" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E220" t="s">
         <v>155</v>
       </c>
       <c r="F220" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="G220" t="s">
         <v>151</v>
@@ -27812,7 +27827,7 @@
         <v>155</v>
       </c>
       <c r="F221" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G221" t="s">
         <v>151</v>
@@ -28133,7 +28148,7 @@
         <v>155</v>
       </c>
       <c r="F224" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G224" t="s">
         <v>69</v>
@@ -28231,7 +28246,7 @@
         <v>415</v>
       </c>
       <c r="C225" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D225" t="s">
         <v>52</v>
@@ -28240,7 +28255,7 @@
         <v>155</v>
       </c>
       <c r="F225" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G225" t="s">
         <v>116</v>
@@ -28549,7 +28564,7 @@
         <v>920</v>
       </c>
       <c r="B228" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="C228" t="s">
         <v>65</v>
@@ -28561,25 +28576,25 @@
         <v>155</v>
       </c>
       <c r="F228" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G228" t="s">
         <v>151</v>
       </c>
       <c r="H228" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="I228" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="J228" t="s">
         <v>84</v>
       </c>
       <c r="K228" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="L228" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="M228" t="s">
         <v>38</v>
@@ -28775,7 +28790,7 @@
         <v>155</v>
       </c>
       <c r="F230" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G230" t="s">
         <v>69</v>
@@ -29738,7 +29753,7 @@
         <v>155</v>
       </c>
       <c r="F239" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G239" t="s">
         <v>116</v>
@@ -29967,7 +29982,7 @@
         <v>84</v>
       </c>
       <c r="K241" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="L241" t="s">
         <v>424</v>
@@ -30374,7 +30389,7 @@
         <v>80</v>
       </c>
       <c r="D245" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="E245" t="s">
         <v>155</v>
@@ -31016,7 +31031,7 @@
         <v>149</v>
       </c>
       <c r="D251" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E251" t="s">
         <v>155</v>
@@ -31236,7 +31251,7 @@
         <v>155</v>
       </c>
       <c r="F253" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G253" t="s">
         <v>116</v>
@@ -32086,7 +32101,7 @@
         <v>299</v>
       </c>
       <c r="D261" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E261" t="s">
         <v>155</v>
@@ -32407,7 +32422,7 @@
         <v>217</v>
       </c>
       <c r="D264" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E264" t="s">
         <v>155</v>
@@ -32511,7 +32526,7 @@
         <v>792</v>
       </c>
       <c r="C265" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D265" t="s">
         <v>52</v>
@@ -32526,7 +32541,7 @@
         <v>69</v>
       </c>
       <c r="H265" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="I265" t="s">
         <v>793</v>
@@ -33263,7 +33278,7 @@
         <v>149</v>
       </c>
       <c r="D272" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E272" t="s">
         <v>155</v>
@@ -34330,7 +34345,7 @@
         <v>704</v>
       </c>
       <c r="C282" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D282" t="s">
         <v>52</v>
@@ -34776,7 +34791,7 @@
         <v>374</v>
       </c>
       <c r="I286" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="J286" t="s">
         <v>43</v>
@@ -34865,7 +34880,7 @@
         <v>587</v>
       </c>
       <c r="C287" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D287" t="s">
         <v>142</v>
@@ -34880,7 +34895,7 @@
         <v>116</v>
       </c>
       <c r="H287" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="I287" t="s">
         <v>588</v>
@@ -34972,7 +34987,7 @@
         <v>856</v>
       </c>
       <c r="C288" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D288" t="s">
         <v>142</v>
@@ -37442,7 +37457,7 @@
         <v>155</v>
       </c>
       <c r="F311" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G311" t="s">
         <v>116</v>
@@ -37977,7 +37992,7 @@
         <v>155</v>
       </c>
       <c r="F316" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G316" t="s">
         <v>69</v>
@@ -38506,13 +38521,13 @@
         <v>303</v>
       </c>
       <c r="D321" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E321" t="s">
         <v>155</v>
       </c>
       <c r="F321" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="G321" t="s">
         <v>151</v>
@@ -39047,7 +39062,7 @@
         <v>155</v>
       </c>
       <c r="F326" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="G326" t="s">
         <v>38</v>
@@ -39261,7 +39276,7 @@
         <v>155</v>
       </c>
       <c r="F328" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G328" t="s">
         <v>116</v>
@@ -39787,7 +39802,7 @@
         <v>1055</v>
       </c>
       <c r="C333" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D333" t="s">
         <v>200</v>
@@ -40117,7 +40132,7 @@
         <v>155</v>
       </c>
       <c r="F336" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G336" t="s">
         <v>69</v>
@@ -40643,7 +40658,7 @@
         <v>1066</v>
       </c>
       <c r="C341" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D341" t="s">
         <v>52</v>
@@ -41074,7 +41089,7 @@
         <v>221</v>
       </c>
       <c r="D345" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="E345" t="s">
         <v>155</v>
@@ -41285,7 +41300,7 @@
         <v>1066</v>
       </c>
       <c r="C347" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D347" t="s">
         <v>52</v>
@@ -42034,7 +42049,7 @@
         <v>1055</v>
       </c>
       <c r="C354" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D354" t="s">
         <v>200</v>
@@ -43747,7 +43762,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -44845,6 +44860,48 @@
         <v>1178</v>
       </c>
     </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>98</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79">
+        <v>387</v>
+      </c>
+      <c r="D79" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>99</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80">
+        <v>389</v>
+      </c>
+      <c r="D80" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>100</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+      <c r="C81">
+        <v>393</v>
+      </c>
+      <c r="D81" t="s">
+        <v>1181</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -44853,7 +44910,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="20" customWidth="1"/>
@@ -44867,19 +44924,19 @@
         <v>1100</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1179</v>
+        <v>1182</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1180</v>
+        <v>1183</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1183</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -44890,19 +44947,19 @@
         <v>379</v>
       </c>
       <c r="C2" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D2" t="s">
         <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -44913,7 +44970,7 @@
         <v>386</v>
       </c>
       <c r="C3" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D3" t="s">
         <v>38</v>
@@ -44925,7 +44982,7 @@
         <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>1187</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -44936,7 +44993,7 @@
         <v>388</v>
       </c>
       <c r="C4" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D4" t="s">
         <v>38</v>
@@ -44948,7 +45005,7 @@
         <v>69</v>
       </c>
       <c r="G4" t="s">
-        <v>1188</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -44959,7 +45016,7 @@
         <v>387</v>
       </c>
       <c r="C5" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D5" t="s">
         <v>38</v>
@@ -44971,7 +45028,7 @@
         <v>69</v>
       </c>
       <c r="G5" t="s">
-        <v>1189</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -44982,7 +45039,7 @@
         <v>388</v>
       </c>
       <c r="C6" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D6" t="s">
         <v>69</v>
@@ -44994,7 +45051,7 @@
         <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>1190</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -45005,19 +45062,19 @@
         <v>387</v>
       </c>
       <c r="C7" t="s">
-        <v>1191</v>
+        <v>1194</v>
       </c>
       <c r="D7" t="s">
         <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>1192</v>
+        <v>1195</v>
       </c>
       <c r="F7" t="s">
         <v>69</v>
       </c>
       <c r="G7" t="s">
-        <v>1193</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -45028,19 +45085,19 @@
         <v>387</v>
       </c>
       <c r="C8" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D8" t="s">
         <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="F8" t="s">
         <v>69</v>
       </c>
       <c r="G8" t="s">
-        <v>1193</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -45051,10 +45108,10 @@
         <v>387</v>
       </c>
       <c r="C9" t="s">
-        <v>1191</v>
+        <v>1194</v>
       </c>
       <c r="D9" t="s">
-        <v>1192</v>
+        <v>1195</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -45063,7 +45120,7 @@
         <v>69</v>
       </c>
       <c r="G9" t="s">
-        <v>1196</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -45074,19 +45131,19 @@
         <v>387</v>
       </c>
       <c r="C10" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D10" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="E10" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="F10" t="s">
         <v>69</v>
       </c>
       <c r="G10" t="s">
-        <v>1198</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -45097,19 +45154,19 @@
         <v>387</v>
       </c>
       <c r="C11" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D11" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="E11" t="s">
-        <v>1199</v>
+        <v>1202</v>
       </c>
       <c r="F11" t="s">
         <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>1200</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -45120,7 +45177,7 @@
         <v>387</v>
       </c>
       <c r="C12" t="s">
-        <v>1191</v>
+        <v>1194</v>
       </c>
       <c r="D12" t="s">
         <v>38</v>
@@ -45132,7 +45189,7 @@
         <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>1201</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -45143,7 +45200,7 @@
         <v>387</v>
       </c>
       <c r="C13" t="s">
-        <v>1202</v>
+        <v>1205</v>
       </c>
       <c r="D13" t="s">
         <v>38</v>
@@ -45155,7 +45212,7 @@
         <v>69</v>
       </c>
       <c r="G13" t="s">
-        <v>1203</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -45166,19 +45223,19 @@
         <v>380</v>
       </c>
       <c r="C14" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D14" t="s">
         <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="F14" t="s">
         <v>69</v>
       </c>
       <c r="G14" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -45189,7 +45246,7 @@
         <v>386</v>
       </c>
       <c r="C15" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D15" t="s">
         <v>38</v>
@@ -45201,7 +45258,7 @@
         <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>1205</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -45212,19 +45269,19 @@
         <v>387</v>
       </c>
       <c r="C16" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D16" t="s">
-        <v>1199</v>
+        <v>1202</v>
       </c>
       <c r="E16" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="F16" t="s">
         <v>69</v>
       </c>
       <c r="G16" t="s">
-        <v>1206</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -45235,10 +45292,10 @@
         <v>387</v>
       </c>
       <c r="C17" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D17" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="E17" t="s">
         <v>109</v>
@@ -45247,7 +45304,7 @@
         <v>69</v>
       </c>
       <c r="G17" t="s">
-        <v>1207</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -45258,7 +45315,7 @@
         <v>387</v>
       </c>
       <c r="C18" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D18" t="s">
         <v>84</v>
@@ -45270,7 +45327,7 @@
         <v>69</v>
       </c>
       <c r="G18" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -45281,7 +45338,7 @@
         <v>387</v>
       </c>
       <c r="C19" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D19" t="s">
         <v>84</v>
@@ -45293,7 +45350,7 @@
         <v>69</v>
       </c>
       <c r="G19" t="s">
-        <v>1209</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -45304,7 +45361,7 @@
         <v>387</v>
       </c>
       <c r="C20" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D20" t="s">
         <v>84</v>
@@ -45316,7 +45373,7 @@
         <v>69</v>
       </c>
       <c r="G20" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -45327,7 +45384,7 @@
         <v>387</v>
       </c>
       <c r="C21" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D21" t="s">
         <v>84</v>
@@ -45339,7 +45396,7 @@
         <v>69</v>
       </c>
       <c r="G21" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -45350,7 +45407,7 @@
         <v>387</v>
       </c>
       <c r="C22" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D22" t="s">
         <v>84</v>
@@ -45362,7 +45419,7 @@
         <v>69</v>
       </c>
       <c r="G22" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -45373,19 +45430,19 @@
         <v>387</v>
       </c>
       <c r="C23" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="D23" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="E23" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="F23" t="s">
         <v>69</v>
       </c>
       <c r="G23" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -45396,10 +45453,10 @@
         <v>387</v>
       </c>
       <c r="C24" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="D24" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="E24" t="s">
         <v>101</v>
@@ -45408,7 +45465,7 @@
         <v>69</v>
       </c>
       <c r="G24" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -45419,7 +45476,7 @@
         <v>387</v>
       </c>
       <c r="C25" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D25" t="s">
         <v>43</v>
@@ -45431,7 +45488,7 @@
         <v>69</v>
       </c>
       <c r="G25" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -45442,19 +45499,19 @@
         <v>386</v>
       </c>
       <c r="C26" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="D26" t="s">
         <v>38</v>
       </c>
       <c r="E26" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="F26" t="s">
         <v>366</v>
       </c>
       <c r="G26" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -45465,7 +45522,7 @@
         <v>391</v>
       </c>
       <c r="C27" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D27" t="s">
         <v>38</v>
@@ -45477,7 +45534,7 @@
         <v>366</v>
       </c>
       <c r="G27" t="s">
-        <v>1219</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -45488,10 +45545,10 @@
         <v>388</v>
       </c>
       <c r="C28" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="D28" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="E28" t="s">
         <v>118</v>
@@ -45500,7 +45557,7 @@
         <v>366</v>
       </c>
       <c r="G28" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -45511,7 +45568,7 @@
         <v>388</v>
       </c>
       <c r="C29" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="D29" t="s">
         <v>43</v>
@@ -45523,7 +45580,7 @@
         <v>366</v>
       </c>
       <c r="G29" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -45534,10 +45591,10 @@
         <v>390</v>
       </c>
       <c r="C30" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="D30" t="s">
-        <v>360</v>
+        <v>343</v>
       </c>
       <c r="E30" t="s">
         <v>69</v>
@@ -45546,7 +45603,7 @@
         <v>69</v>
       </c>
       <c r="G30" t="s">
-        <v>1223</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -45557,10 +45614,10 @@
         <v>391</v>
       </c>
       <c r="C31" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="D31" t="s">
-        <v>360</v>
+        <v>343</v>
       </c>
       <c r="E31" t="s">
         <v>69</v>
@@ -45569,7 +45626,7 @@
         <v>69</v>
       </c>
       <c r="G31" t="s">
-        <v>1224</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -45580,10 +45637,10 @@
         <v>381</v>
       </c>
       <c r="C32" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="D32" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E32" t="s">
         <v>116</v>
@@ -45592,7 +45649,7 @@
         <v>116</v>
       </c>
       <c r="G32" t="s">
-        <v>1225</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -45603,10 +45660,10 @@
         <v>381</v>
       </c>
       <c r="C33" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="D33" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E33" t="s">
         <v>38</v>
@@ -45615,7 +45672,7 @@
         <v>69</v>
       </c>
       <c r="G33" t="s">
-        <v>1227</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -45626,10 +45683,10 @@
         <v>391</v>
       </c>
       <c r="C34" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="D34" t="s">
-        <v>360</v>
+        <v>343</v>
       </c>
       <c r="E34" t="s">
         <v>38</v>
@@ -45638,7 +45695,7 @@
         <v>69</v>
       </c>
       <c r="G34" t="s">
-        <v>1228</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -45649,10 +45706,10 @@
         <v>390</v>
       </c>
       <c r="C35" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="D35" t="s">
-        <v>360</v>
+        <v>343</v>
       </c>
       <c r="E35" t="s">
         <v>38</v>
@@ -45661,7 +45718,7 @@
         <v>69</v>
       </c>
       <c r="G35" t="s">
-        <v>1229</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -45672,7 +45729,7 @@
         <v>385</v>
       </c>
       <c r="C36" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -45684,7 +45741,7 @@
         <v>151</v>
       </c>
       <c r="G36" t="s">
-        <v>1230</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -45695,7 +45752,7 @@
         <v>392</v>
       </c>
       <c r="C37" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D37" t="s">
         <v>38</v>
@@ -45707,7 +45764,7 @@
         <v>151</v>
       </c>
       <c r="G37" t="s">
-        <v>1231</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -45718,7 +45775,7 @@
         <v>382</v>
       </c>
       <c r="C38" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="D38" t="s">
         <v>38</v>
@@ -45730,7 +45787,7 @@
         <v>151</v>
       </c>
       <c r="G38" t="s">
-        <v>1232</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -45741,19 +45798,65 @@
         <v>392</v>
       </c>
       <c r="C39" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="D39" t="s">
         <v>38</v>
       </c>
       <c r="E39" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="F39" t="s">
         <v>69</v>
       </c>
       <c r="G39" t="s">
-        <v>1233</v>
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>389</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D40" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" t="s">
+        <v>69</v>
+      </c>
+      <c r="F40" t="s">
+        <v>69</v>
+      </c>
+      <c r="G40" t="s">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>393</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" t="s">
+        <v>69</v>
+      </c>
+      <c r="F41" t="s">
+        <v>69</v>
+      </c>
+      <c r="G41" t="s">
+        <v>1238</v>
       </c>
     </row>
   </sheetData>
@@ -45775,16 +45878,16 @@
         <v>1098</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1234</v>
+        <v>1239</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1235</v>
+        <v>1240</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1100</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1236</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -45792,16 +45895,16 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>1237</v>
+        <v>1242</v>
       </c>
       <c r="C2" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D2">
         <v>380</v>
       </c>
       <c r="E2" t="s">
-        <v>1239</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -45809,16 +45912,16 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>1240</v>
+        <v>1245</v>
       </c>
       <c r="C3" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D3">
         <v>381</v>
       </c>
       <c r="E3" t="s">
-        <v>1241</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -45826,16 +45929,16 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>1242</v>
+        <v>1247</v>
       </c>
       <c r="C4" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D4">
         <v>382</v>
       </c>
       <c r="E4" t="s">
-        <v>1243</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -45843,16 +45946,16 @@
         <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>1244</v>
+        <v>1249</v>
       </c>
       <c r="C5" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D5">
         <v>383</v>
       </c>
       <c r="E5" t="s">
-        <v>1245</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -45860,16 +45963,16 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>1246</v>
+        <v>1251</v>
       </c>
       <c r="C6" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D6">
         <v>385</v>
       </c>
       <c r="E6" t="s">
-        <v>1247</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -45877,16 +45980,16 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>1248</v>
+        <v>1253</v>
       </c>
       <c r="C7" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D7">
         <v>386</v>
       </c>
       <c r="E7" t="s">
-        <v>1249</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -45894,16 +45997,16 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>1250</v>
+        <v>1255</v>
       </c>
       <c r="C8" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D8">
         <v>387</v>
       </c>
       <c r="E8" t="s">
-        <v>1251</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -45911,16 +46014,16 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>1252</v>
+        <v>1257</v>
       </c>
       <c r="C9" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D9">
         <v>388</v>
       </c>
       <c r="E9" t="s">
-        <v>1253</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -45928,16 +46031,16 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>1254</v>
+        <v>1259</v>
       </c>
       <c r="C10" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D10">
         <v>389</v>
       </c>
       <c r="E10" t="s">
-        <v>1255</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -45945,16 +46048,16 @@
         <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>1256</v>
+        <v>1261</v>
       </c>
       <c r="C11" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D11">
         <v>390</v>
       </c>
       <c r="E11" t="s">
-        <v>1257</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -45962,16 +46065,16 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>1258</v>
+        <v>1263</v>
       </c>
       <c r="C12" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D12">
         <v>391</v>
       </c>
       <c r="E12" t="s">
-        <v>1259</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -45979,16 +46082,16 @@
         <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>1260</v>
+        <v>1265</v>
       </c>
       <c r="C13" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D13">
         <v>392</v>
       </c>
       <c r="E13" t="s">
-        <v>1261</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -45996,16 +46099,16 @@
         <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>1262</v>
+        <v>1267</v>
       </c>
       <c r="C14" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D14">
         <v>393</v>
       </c>
       <c r="E14" t="s">
-        <v>1263</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -46013,16 +46116,16 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>1264</v>
+        <v>1269</v>
       </c>
       <c r="C15" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D15">
         <v>384</v>
       </c>
       <c r="E15" t="s">
-        <v>1265</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -46030,16 +46133,16 @@
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>1266</v>
+        <v>1271</v>
       </c>
       <c r="C16" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D16">
         <v>394</v>
       </c>
       <c r="E16" t="s">
-        <v>1267</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -46047,16 +46150,16 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>1268</v>
+        <v>1273</v>
       </c>
       <c r="C17" t="s">
-        <v>1238</v>
+        <v>1243</v>
       </c>
       <c r="D17">
         <v>395</v>
       </c>
       <c r="E17" t="s">
-        <v>1269</v>
+        <v>1274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>